<commit_message>
Add PCDS dates for  biomass readings
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/WaggaWagga2024/DookieWaggaWagga2024.xlsx
+++ b/Tests/Validation/Wheat/WaggaWagga2024/DookieWaggaWagga2024.xlsx
@@ -200,7 +200,46 @@
     <t xml:space="preserve">20/11/2024 00:00:00</t>
   </si>
   <si>
-    <t xml:space="preserve">28/08/2024 00:00:00</t>
+    <t xml:space="preserve">09/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05/10/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07/10/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/10/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08/10/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/09/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01/10/2024 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02/10/2024 00:00:00</t>
   </si>
   <si>
     <t xml:space="preserve">29/04/2024 00:00:00</t>
@@ -230,22 +269,13 @@
     <t xml:space="preserve">07/06/2024 00:00:00</t>
   </si>
   <si>
+    <t xml:space="preserve">28/08/2024 00:00:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">02/09/2024 00:00:00</t>
   </si>
   <si>
-    <t xml:space="preserve">06/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09/09/2024 00:00:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">16/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02/10/2024 00:00:00</t>
   </si>
   <si>
     <t xml:space="preserve">10/10/2024 00:00:00</t>
@@ -255,36 +285,6 @@
   </si>
   <si>
     <t xml:space="preserve">01/05/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07/09/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05/10/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07/10/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04/10/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08/10/2024 00:00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01/10/2024 00:00:00</t>
   </si>
 </sst>
 </file>
@@ -20910,7 +20910,7 @@
         <v>21</v>
       </c>
       <c r="B755" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C755"/>
       <c r="D755"/>
@@ -20962,7 +20962,7 @@
         <v>23</v>
       </c>
       <c r="B757" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C757"/>
       <c r="D757"/>
@@ -20989,7 +20989,7 @@
         <v>24</v>
       </c>
       <c r="B758" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C758"/>
       <c r="D758"/>
@@ -21014,7 +21014,7 @@
         <v>25</v>
       </c>
       <c r="B759" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C759"/>
       <c r="D759"/>
@@ -21041,7 +21041,7 @@
         <v>26</v>
       </c>
       <c r="B760" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C760"/>
       <c r="D760"/>
@@ -21068,7 +21068,7 @@
         <v>27</v>
       </c>
       <c r="B761" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C761"/>
       <c r="D761"/>
@@ -21095,7 +21095,7 @@
         <v>28</v>
       </c>
       <c r="B762" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C762"/>
       <c r="D762"/>
@@ -21122,7 +21122,7 @@
         <v>29</v>
       </c>
       <c r="B763" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C763"/>
       <c r="D763"/>
@@ -21149,7 +21149,7 @@
         <v>30</v>
       </c>
       <c r="B764" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C764"/>
       <c r="D764"/>
@@ -21176,7 +21176,7 @@
         <v>31</v>
       </c>
       <c r="B765" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C765"/>
       <c r="D765"/>
@@ -21203,7 +21203,7 @@
         <v>32</v>
       </c>
       <c r="B766" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C766"/>
       <c r="D766"/>
@@ -21230,7 +21230,7 @@
         <v>33</v>
       </c>
       <c r="B767" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C767"/>
       <c r="D767"/>
@@ -21284,7 +21284,7 @@
         <v>35</v>
       </c>
       <c r="B769" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C769"/>
       <c r="D769"/>
@@ -21311,7 +21311,7 @@
         <v>19</v>
       </c>
       <c r="B770" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C770"/>
       <c r="D770"/>
@@ -21338,7 +21338,7 @@
         <v>21</v>
       </c>
       <c r="B771" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C771"/>
       <c r="D771"/>
@@ -21365,7 +21365,7 @@
         <v>22</v>
       </c>
       <c r="B772" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C772"/>
       <c r="D772"/>
@@ -21392,7 +21392,7 @@
         <v>23</v>
       </c>
       <c r="B773" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C773"/>
       <c r="D773"/>
@@ -21419,7 +21419,7 @@
         <v>24</v>
       </c>
       <c r="B774" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C774"/>
       <c r="D774"/>
@@ -21446,7 +21446,7 @@
         <v>25</v>
       </c>
       <c r="B775" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C775"/>
       <c r="D775"/>
@@ -21473,7 +21473,7 @@
         <v>26</v>
       </c>
       <c r="B776" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C776"/>
       <c r="D776"/>
@@ -21500,7 +21500,7 @@
         <v>27</v>
       </c>
       <c r="B777" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C777"/>
       <c r="D777"/>
@@ -21527,7 +21527,7 @@
         <v>28</v>
       </c>
       <c r="B778" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C778"/>
       <c r="D778"/>
@@ -21554,7 +21554,7 @@
         <v>29</v>
       </c>
       <c r="B779" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C779"/>
       <c r="D779"/>
@@ -21581,7 +21581,7 @@
         <v>30</v>
       </c>
       <c r="B780" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C780"/>
       <c r="D780"/>
@@ -21608,7 +21608,7 @@
         <v>31</v>
       </c>
       <c r="B781" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C781"/>
       <c r="D781"/>
@@ -21635,7 +21635,7 @@
         <v>32</v>
       </c>
       <c r="B782" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C782"/>
       <c r="D782"/>
@@ -21662,7 +21662,7 @@
         <v>33</v>
       </c>
       <c r="B783" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C783"/>
       <c r="D783"/>
@@ -21689,7 +21689,7 @@
         <v>34</v>
       </c>
       <c r="B784" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C784"/>
       <c r="D784"/>
@@ -21716,7 +21716,7 @@
         <v>35</v>
       </c>
       <c r="B785" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C785"/>
       <c r="D785"/>
@@ -22202,7 +22202,7 @@
         <v>21</v>
       </c>
       <c r="B803" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C803"/>
       <c r="D803"/>
@@ -22254,7 +22254,7 @@
         <v>23</v>
       </c>
       <c r="B805" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C805"/>
       <c r="D805"/>
@@ -22281,7 +22281,7 @@
         <v>24</v>
       </c>
       <c r="B806" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C806"/>
       <c r="D806"/>
@@ -22306,7 +22306,7 @@
         <v>25</v>
       </c>
       <c r="B807" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C807"/>
       <c r="D807"/>
@@ -22333,7 +22333,7 @@
         <v>26</v>
       </c>
       <c r="B808" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C808"/>
       <c r="D808"/>
@@ -22360,7 +22360,7 @@
         <v>27</v>
       </c>
       <c r="B809" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C809"/>
       <c r="D809"/>
@@ -22387,7 +22387,7 @@
         <v>28</v>
       </c>
       <c r="B810" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C810"/>
       <c r="D810"/>
@@ -22414,7 +22414,7 @@
         <v>29</v>
       </c>
       <c r="B811" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C811"/>
       <c r="D811"/>
@@ -22441,7 +22441,7 @@
         <v>30</v>
       </c>
       <c r="B812" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C812"/>
       <c r="D812"/>
@@ -22468,7 +22468,7 @@
         <v>31</v>
       </c>
       <c r="B813" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C813"/>
       <c r="D813"/>
@@ -22495,7 +22495,7 @@
         <v>32</v>
       </c>
       <c r="B814" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C814"/>
       <c r="D814"/>
@@ -22522,7 +22522,7 @@
         <v>33</v>
       </c>
       <c r="B815" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C815"/>
       <c r="D815"/>
@@ -22576,7 +22576,7 @@
         <v>35</v>
       </c>
       <c r="B817" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C817"/>
       <c r="D817"/>
@@ -22603,7 +22603,7 @@
         <v>19</v>
       </c>
       <c r="B818" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C818"/>
       <c r="D818"/>
@@ -22630,7 +22630,7 @@
         <v>21</v>
       </c>
       <c r="B819" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C819"/>
       <c r="D819"/>
@@ -22657,7 +22657,7 @@
         <v>22</v>
       </c>
       <c r="B820" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C820"/>
       <c r="D820"/>
@@ -22684,7 +22684,7 @@
         <v>23</v>
       </c>
       <c r="B821" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C821"/>
       <c r="D821"/>
@@ -22711,7 +22711,7 @@
         <v>24</v>
       </c>
       <c r="B822" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C822"/>
       <c r="D822"/>
@@ -22738,7 +22738,7 @@
         <v>25</v>
       </c>
       <c r="B823" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C823"/>
       <c r="D823"/>
@@ -22765,7 +22765,7 @@
         <v>26</v>
       </c>
       <c r="B824" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C824"/>
       <c r="D824"/>
@@ -22792,7 +22792,7 @@
         <v>27</v>
       </c>
       <c r="B825" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C825"/>
       <c r="D825"/>
@@ -22819,7 +22819,7 @@
         <v>28</v>
       </c>
       <c r="B826" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C826"/>
       <c r="D826"/>
@@ -22846,7 +22846,7 @@
         <v>29</v>
       </c>
       <c r="B827" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C827"/>
       <c r="D827"/>
@@ -22873,7 +22873,7 @@
         <v>30</v>
       </c>
       <c r="B828" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C828"/>
       <c r="D828"/>
@@ -22900,7 +22900,7 @@
         <v>31</v>
       </c>
       <c r="B829" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C829"/>
       <c r="D829"/>
@@ -22927,7 +22927,7 @@
         <v>32</v>
       </c>
       <c r="B830" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C830"/>
       <c r="D830"/>
@@ -22954,7 +22954,7 @@
         <v>33</v>
       </c>
       <c r="B831" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C831"/>
       <c r="D831"/>
@@ -22981,7 +22981,7 @@
         <v>34</v>
       </c>
       <c r="B832" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C832"/>
       <c r="D832"/>
@@ -23008,7 +23008,7 @@
         <v>35</v>
       </c>
       <c r="B833" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C833"/>
       <c r="D833"/>
@@ -23494,7 +23494,7 @@
         <v>21</v>
       </c>
       <c r="B851" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C851"/>
       <c r="D851"/>
@@ -23546,7 +23546,7 @@
         <v>23</v>
       </c>
       <c r="B853" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C853"/>
       <c r="D853"/>
@@ -23573,7 +23573,7 @@
         <v>24</v>
       </c>
       <c r="B854" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C854"/>
       <c r="D854"/>
@@ -23598,7 +23598,7 @@
         <v>25</v>
       </c>
       <c r="B855" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C855"/>
       <c r="D855"/>
@@ -23625,7 +23625,7 @@
         <v>26</v>
       </c>
       <c r="B856" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C856"/>
       <c r="D856"/>
@@ -23652,7 +23652,7 @@
         <v>27</v>
       </c>
       <c r="B857" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C857"/>
       <c r="D857"/>
@@ -23679,7 +23679,7 @@
         <v>28</v>
       </c>
       <c r="B858" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C858"/>
       <c r="D858"/>
@@ -23706,7 +23706,7 @@
         <v>29</v>
       </c>
       <c r="B859" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C859"/>
       <c r="D859"/>
@@ -23733,7 +23733,7 @@
         <v>30</v>
       </c>
       <c r="B860" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C860"/>
       <c r="D860"/>
@@ -23760,7 +23760,7 @@
         <v>31</v>
       </c>
       <c r="B861" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C861"/>
       <c r="D861"/>
@@ -23787,7 +23787,7 @@
         <v>32</v>
       </c>
       <c r="B862" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C862"/>
       <c r="D862"/>
@@ -23814,7 +23814,7 @@
         <v>33</v>
       </c>
       <c r="B863" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C863"/>
       <c r="D863"/>
@@ -23868,7 +23868,7 @@
         <v>35</v>
       </c>
       <c r="B865" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C865"/>
       <c r="D865"/>
@@ -23895,7 +23895,7 @@
         <v>19</v>
       </c>
       <c r="B866" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C866"/>
       <c r="D866"/>
@@ -23922,7 +23922,7 @@
         <v>21</v>
       </c>
       <c r="B867" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C867"/>
       <c r="D867"/>
@@ -23949,7 +23949,7 @@
         <v>22</v>
       </c>
       <c r="B868" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C868"/>
       <c r="D868"/>
@@ -23976,7 +23976,7 @@
         <v>23</v>
       </c>
       <c r="B869" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C869"/>
       <c r="D869"/>
@@ -24003,7 +24003,7 @@
         <v>24</v>
       </c>
       <c r="B870" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C870"/>
       <c r="D870"/>
@@ -24030,7 +24030,7 @@
         <v>25</v>
       </c>
       <c r="B871" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C871"/>
       <c r="D871"/>
@@ -24057,7 +24057,7 @@
         <v>26</v>
       </c>
       <c r="B872" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C872"/>
       <c r="D872"/>
@@ -24084,7 +24084,7 @@
         <v>27</v>
       </c>
       <c r="B873" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C873"/>
       <c r="D873"/>
@@ -24111,7 +24111,7 @@
         <v>28</v>
       </c>
       <c r="B874" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C874"/>
       <c r="D874"/>
@@ -24138,7 +24138,7 @@
         <v>29</v>
       </c>
       <c r="B875" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C875"/>
       <c r="D875"/>
@@ -24165,7 +24165,7 @@
         <v>30</v>
       </c>
       <c r="B876" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C876"/>
       <c r="D876"/>
@@ -24192,7 +24192,7 @@
         <v>31</v>
       </c>
       <c r="B877" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C877"/>
       <c r="D877"/>
@@ -24219,7 +24219,7 @@
         <v>32</v>
       </c>
       <c r="B878" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C878"/>
       <c r="D878"/>
@@ -24246,7 +24246,7 @@
         <v>33</v>
       </c>
       <c r="B879" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C879"/>
       <c r="D879"/>
@@ -24273,7 +24273,7 @@
         <v>34</v>
       </c>
       <c r="B880" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C880"/>
       <c r="D880"/>
@@ -24300,7 +24300,7 @@
         <v>35</v>
       </c>
       <c r="B881" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C881"/>
       <c r="D881"/>
@@ -24786,7 +24786,7 @@
         <v>21</v>
       </c>
       <c r="B899" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C899"/>
       <c r="D899"/>
@@ -24838,7 +24838,7 @@
         <v>23</v>
       </c>
       <c r="B901" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C901"/>
       <c r="D901"/>
@@ -24865,7 +24865,7 @@
         <v>24</v>
       </c>
       <c r="B902" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C902"/>
       <c r="D902"/>
@@ -24890,7 +24890,7 @@
         <v>25</v>
       </c>
       <c r="B903" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C903"/>
       <c r="D903"/>
@@ -24917,7 +24917,7 @@
         <v>26</v>
       </c>
       <c r="B904" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C904"/>
       <c r="D904"/>
@@ -24944,7 +24944,7 @@
         <v>27</v>
       </c>
       <c r="B905" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C905"/>
       <c r="D905"/>
@@ -24971,7 +24971,7 @@
         <v>28</v>
       </c>
       <c r="B906" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C906"/>
       <c r="D906"/>
@@ -24998,7 +24998,7 @@
         <v>29</v>
       </c>
       <c r="B907" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C907"/>
       <c r="D907"/>
@@ -25025,7 +25025,7 @@
         <v>30</v>
       </c>
       <c r="B908" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C908"/>
       <c r="D908"/>
@@ -25052,7 +25052,7 @@
         <v>31</v>
       </c>
       <c r="B909" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C909"/>
       <c r="D909"/>
@@ -25079,7 +25079,7 @@
         <v>32</v>
       </c>
       <c r="B910" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C910"/>
       <c r="D910"/>
@@ -25106,7 +25106,7 @@
         <v>33</v>
       </c>
       <c r="B911" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C911"/>
       <c r="D911"/>
@@ -25160,7 +25160,7 @@
         <v>35</v>
       </c>
       <c r="B913" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C913"/>
       <c r="D913"/>
@@ -25187,7 +25187,7 @@
         <v>19</v>
       </c>
       <c r="B914" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C914"/>
       <c r="D914"/>
@@ -25214,7 +25214,7 @@
         <v>21</v>
       </c>
       <c r="B915" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C915"/>
       <c r="D915"/>
@@ -25241,7 +25241,7 @@
         <v>22</v>
       </c>
       <c r="B916" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C916"/>
       <c r="D916"/>
@@ -25268,7 +25268,7 @@
         <v>23</v>
       </c>
       <c r="B917" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C917"/>
       <c r="D917"/>
@@ -25295,7 +25295,7 @@
         <v>24</v>
       </c>
       <c r="B918" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C918"/>
       <c r="D918"/>
@@ -25322,7 +25322,7 @@
         <v>25</v>
       </c>
       <c r="B919" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C919"/>
       <c r="D919"/>
@@ -25349,7 +25349,7 @@
         <v>26</v>
       </c>
       <c r="B920" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C920"/>
       <c r="D920"/>
@@ -25376,7 +25376,7 @@
         <v>27</v>
       </c>
       <c r="B921" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C921"/>
       <c r="D921"/>
@@ -25403,7 +25403,7 @@
         <v>28</v>
       </c>
       <c r="B922" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C922"/>
       <c r="D922"/>
@@ -25430,7 +25430,7 @@
         <v>29</v>
       </c>
       <c r="B923" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C923"/>
       <c r="D923"/>
@@ -25457,7 +25457,7 @@
         <v>30</v>
       </c>
       <c r="B924" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C924"/>
       <c r="D924"/>
@@ -25484,7 +25484,7 @@
         <v>31</v>
       </c>
       <c r="B925" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C925"/>
       <c r="D925"/>
@@ -25511,7 +25511,7 @@
         <v>32</v>
       </c>
       <c r="B926" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C926"/>
       <c r="D926"/>
@@ -25538,7 +25538,7 @@
         <v>33</v>
       </c>
       <c r="B927" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C927"/>
       <c r="D927"/>
@@ -25565,7 +25565,7 @@
         <v>34</v>
       </c>
       <c r="B928" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C928"/>
       <c r="D928"/>
@@ -25592,7 +25592,7 @@
         <v>35</v>
       </c>
       <c r="B929" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C929"/>
       <c r="D929"/>
@@ -25646,7 +25646,7 @@
         <v>21</v>
       </c>
       <c r="B931" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C931"/>
       <c r="D931"/>
@@ -25698,7 +25698,7 @@
         <v>23</v>
       </c>
       <c r="B933" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C933"/>
       <c r="D933"/>
@@ -25725,7 +25725,7 @@
         <v>24</v>
       </c>
       <c r="B934" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C934"/>
       <c r="D934"/>
@@ -25750,7 +25750,7 @@
         <v>25</v>
       </c>
       <c r="B935" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C935"/>
       <c r="D935"/>
@@ -25777,7 +25777,7 @@
         <v>26</v>
       </c>
       <c r="B936" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C936"/>
       <c r="D936"/>
@@ -25804,7 +25804,7 @@
         <v>27</v>
       </c>
       <c r="B937" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C937"/>
       <c r="D937"/>
@@ -25831,7 +25831,7 @@
         <v>28</v>
       </c>
       <c r="B938" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C938"/>
       <c r="D938"/>
@@ -25858,7 +25858,7 @@
         <v>29</v>
       </c>
       <c r="B939" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C939"/>
       <c r="D939"/>
@@ -25885,7 +25885,7 @@
         <v>30</v>
       </c>
       <c r="B940" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C940"/>
       <c r="D940"/>
@@ -25912,7 +25912,7 @@
         <v>31</v>
       </c>
       <c r="B941" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C941"/>
       <c r="D941"/>
@@ -25939,7 +25939,7 @@
         <v>32</v>
       </c>
       <c r="B942" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C942"/>
       <c r="D942"/>
@@ -25966,7 +25966,7 @@
         <v>33</v>
       </c>
       <c r="B943" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C943"/>
       <c r="D943"/>
@@ -26020,7 +26020,7 @@
         <v>35</v>
       </c>
       <c r="B945" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C945"/>
       <c r="D945"/>
@@ -26047,7 +26047,7 @@
         <v>19</v>
       </c>
       <c r="B946" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C946"/>
       <c r="D946"/>
@@ -26072,7 +26072,7 @@
         <v>21</v>
       </c>
       <c r="B947" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C947"/>
       <c r="D947"/>
@@ -26097,7 +26097,7 @@
         <v>22</v>
       </c>
       <c r="B948" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C948"/>
       <c r="D948"/>
@@ -26122,7 +26122,7 @@
         <v>23</v>
       </c>
       <c r="B949" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C949"/>
       <c r="D949"/>
@@ -26147,7 +26147,7 @@
         <v>24</v>
       </c>
       <c r="B950" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C950"/>
       <c r="D950"/>
@@ -26172,7 +26172,7 @@
         <v>25</v>
       </c>
       <c r="B951" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C951"/>
       <c r="D951"/>
@@ -26197,7 +26197,7 @@
         <v>26</v>
       </c>
       <c r="B952" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C952"/>
       <c r="D952"/>
@@ -26222,7 +26222,7 @@
         <v>27</v>
       </c>
       <c r="B953" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C953"/>
       <c r="D953"/>
@@ -26247,7 +26247,7 @@
         <v>28</v>
       </c>
       <c r="B954" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C954"/>
       <c r="D954"/>
@@ -26272,7 +26272,7 @@
         <v>29</v>
       </c>
       <c r="B955" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C955"/>
       <c r="D955"/>
@@ -26297,7 +26297,7 @@
         <v>30</v>
       </c>
       <c r="B956" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C956"/>
       <c r="D956"/>
@@ -26322,7 +26322,7 @@
         <v>31</v>
       </c>
       <c r="B957" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C957"/>
       <c r="D957"/>
@@ -26347,7 +26347,7 @@
         <v>32</v>
       </c>
       <c r="B958" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C958"/>
       <c r="D958"/>
@@ -26372,7 +26372,7 @@
         <v>33</v>
       </c>
       <c r="B959" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C959"/>
       <c r="D959"/>
@@ -26397,7 +26397,7 @@
         <v>34</v>
       </c>
       <c r="B960" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C960"/>
       <c r="D960"/>
@@ -26422,7 +26422,7 @@
         <v>35</v>
       </c>
       <c r="B961" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C961"/>
       <c r="D961"/>
@@ -26906,7 +26906,7 @@
         <v>21</v>
       </c>
       <c r="B979" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C979"/>
       <c r="D979"/>
@@ -26960,7 +26960,7 @@
         <v>23</v>
       </c>
       <c r="B981" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C981"/>
       <c r="D981"/>
@@ -26987,7 +26987,7 @@
         <v>24</v>
       </c>
       <c r="B982" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C982"/>
       <c r="D982"/>
@@ -27014,7 +27014,7 @@
         <v>25</v>
       </c>
       <c r="B983" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C983"/>
       <c r="D983"/>
@@ -27041,7 +27041,7 @@
         <v>26</v>
       </c>
       <c r="B984" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C984"/>
       <c r="D984"/>
@@ -27068,7 +27068,7 @@
         <v>27</v>
       </c>
       <c r="B985" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C985"/>
       <c r="D985"/>
@@ -27095,7 +27095,7 @@
         <v>28</v>
       </c>
       <c r="B986" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C986"/>
       <c r="D986"/>
@@ -27122,7 +27122,7 @@
         <v>29</v>
       </c>
       <c r="B987" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C987"/>
       <c r="D987"/>
@@ -27149,7 +27149,7 @@
         <v>30</v>
       </c>
       <c r="B988" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C988"/>
       <c r="D988"/>
@@ -27176,7 +27176,7 @@
         <v>31</v>
       </c>
       <c r="B989" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C989"/>
       <c r="D989"/>
@@ -27203,7 +27203,7 @@
         <v>32</v>
       </c>
       <c r="B990" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C990"/>
       <c r="D990"/>
@@ -27230,7 +27230,7 @@
         <v>33</v>
       </c>
       <c r="B991" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C991"/>
       <c r="D991"/>
@@ -27284,7 +27284,7 @@
         <v>35</v>
       </c>
       <c r="B993" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C993"/>
       <c r="D993"/>
@@ -27311,7 +27311,7 @@
         <v>19</v>
       </c>
       <c r="B994" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C994"/>
       <c r="D994"/>
@@ -27338,7 +27338,7 @@
         <v>21</v>
       </c>
       <c r="B995" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C995"/>
       <c r="D995"/>
@@ -27365,7 +27365,7 @@
         <v>22</v>
       </c>
       <c r="B996" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C996"/>
       <c r="D996"/>
@@ -27392,7 +27392,7 @@
         <v>23</v>
       </c>
       <c r="B997" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C997"/>
       <c r="D997"/>
@@ -27419,7 +27419,7 @@
         <v>24</v>
       </c>
       <c r="B998" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C998"/>
       <c r="D998"/>
@@ -27446,7 +27446,7 @@
         <v>25</v>
       </c>
       <c r="B999" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C999"/>
       <c r="D999"/>
@@ -27473,7 +27473,7 @@
         <v>26</v>
       </c>
       <c r="B1000" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C1000"/>
       <c r="D1000"/>
@@ -27500,7 +27500,7 @@
         <v>27</v>
       </c>
       <c r="B1001" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C1001"/>
       <c r="D1001"/>
@@ -27527,7 +27527,7 @@
         <v>28</v>
       </c>
       <c r="B1002" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C1002"/>
       <c r="D1002"/>
@@ -27554,7 +27554,7 @@
         <v>29</v>
       </c>
       <c r="B1003" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C1003"/>
       <c r="D1003"/>
@@ -27581,7 +27581,7 @@
         <v>30</v>
       </c>
       <c r="B1004" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C1004"/>
       <c r="D1004"/>
@@ -27608,7 +27608,7 @@
         <v>31</v>
       </c>
       <c r="B1005" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C1005"/>
       <c r="D1005"/>
@@ -27635,7 +27635,7 @@
         <v>32</v>
       </c>
       <c r="B1006" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C1006"/>
       <c r="D1006"/>
@@ -27662,7 +27662,7 @@
         <v>33</v>
       </c>
       <c r="B1007" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C1007"/>
       <c r="D1007"/>
@@ -27689,7 +27689,7 @@
         <v>34</v>
       </c>
       <c r="B1008" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C1008"/>
       <c r="D1008"/>
@@ -27716,7 +27716,7 @@
         <v>35</v>
       </c>
       <c r="B1009" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C1009"/>
       <c r="D1009"/>
@@ -27743,7 +27743,7 @@
         <v>19</v>
       </c>
       <c r="B1010" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1010"/>
       <c r="D1010"/>
@@ -27768,7 +27768,7 @@
         <v>21</v>
       </c>
       <c r="B1011" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1011"/>
       <c r="D1011"/>
@@ -27795,7 +27795,7 @@
         <v>22</v>
       </c>
       <c r="B1012" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1012"/>
       <c r="D1012"/>
@@ -27822,7 +27822,7 @@
         <v>23</v>
       </c>
       <c r="B1013" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1013"/>
       <c r="D1013"/>
@@ -27847,7 +27847,7 @@
         <v>24</v>
       </c>
       <c r="B1014" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1014"/>
       <c r="D1014"/>
@@ -27874,7 +27874,7 @@
         <v>25</v>
       </c>
       <c r="B1015" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1015"/>
       <c r="D1015"/>
@@ -27899,7 +27899,7 @@
         <v>26</v>
       </c>
       <c r="B1016" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1016"/>
       <c r="D1016"/>
@@ -27924,7 +27924,7 @@
         <v>27</v>
       </c>
       <c r="B1017" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1017"/>
       <c r="D1017"/>
@@ -27951,7 +27951,7 @@
         <v>28</v>
       </c>
       <c r="B1018" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1018"/>
       <c r="D1018"/>
@@ -27978,7 +27978,7 @@
         <v>29</v>
       </c>
       <c r="B1019" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1019"/>
       <c r="D1019"/>
@@ -28005,7 +28005,7 @@
         <v>30</v>
       </c>
       <c r="B1020" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1020"/>
       <c r="D1020"/>
@@ -28030,7 +28030,7 @@
         <v>31</v>
       </c>
       <c r="B1021" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1021"/>
       <c r="D1021"/>
@@ -28055,7 +28055,7 @@
         <v>32</v>
       </c>
       <c r="B1022" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1022"/>
       <c r="D1022"/>
@@ -28082,7 +28082,7 @@
         <v>33</v>
       </c>
       <c r="B1023" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1023"/>
       <c r="D1023"/>
@@ -28107,7 +28107,7 @@
         <v>34</v>
       </c>
       <c r="B1024" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1024"/>
       <c r="D1024"/>
@@ -28134,7 +28134,7 @@
         <v>35</v>
       </c>
       <c r="B1025" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C1025"/>
       <c r="D1025"/>
@@ -28159,7 +28159,7 @@
         <v>19</v>
       </c>
       <c r="B1026" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1026"/>
       <c r="D1026"/>
@@ -28184,7 +28184,7 @@
         <v>21</v>
       </c>
       <c r="B1027" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1027"/>
       <c r="D1027"/>
@@ -28211,7 +28211,7 @@
         <v>22</v>
       </c>
       <c r="B1028" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1028"/>
       <c r="D1028"/>
@@ -28238,7 +28238,7 @@
         <v>23</v>
       </c>
       <c r="B1029" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1029"/>
       <c r="D1029"/>
@@ -28263,7 +28263,7 @@
         <v>24</v>
       </c>
       <c r="B1030" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1030"/>
       <c r="D1030"/>
@@ -28290,7 +28290,7 @@
         <v>25</v>
       </c>
       <c r="B1031" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1031"/>
       <c r="D1031"/>
@@ -28315,7 +28315,7 @@
         <v>26</v>
       </c>
       <c r="B1032" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1032"/>
       <c r="D1032"/>
@@ -28340,7 +28340,7 @@
         <v>27</v>
       </c>
       <c r="B1033" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1033"/>
       <c r="D1033"/>
@@ -28367,7 +28367,7 @@
         <v>28</v>
       </c>
       <c r="B1034" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1034"/>
       <c r="D1034"/>
@@ -28394,7 +28394,7 @@
         <v>29</v>
       </c>
       <c r="B1035" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1035"/>
       <c r="D1035"/>
@@ -28421,7 +28421,7 @@
         <v>30</v>
       </c>
       <c r="B1036" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1036"/>
       <c r="D1036"/>
@@ -28446,7 +28446,7 @@
         <v>31</v>
       </c>
       <c r="B1037" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1037"/>
       <c r="D1037"/>
@@ -28471,7 +28471,7 @@
         <v>32</v>
       </c>
       <c r="B1038" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1038"/>
       <c r="D1038"/>
@@ -28498,7 +28498,7 @@
         <v>33</v>
       </c>
       <c r="B1039" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1039"/>
       <c r="D1039"/>
@@ -28523,7 +28523,7 @@
         <v>34</v>
       </c>
       <c r="B1040" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1040"/>
       <c r="D1040"/>
@@ -28550,7 +28550,7 @@
         <v>35</v>
       </c>
       <c r="B1041" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C1041"/>
       <c r="D1041"/>
@@ -28575,7 +28575,7 @@
         <v>19</v>
       </c>
       <c r="B1042" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1042"/>
       <c r="D1042"/>
@@ -28600,7 +28600,7 @@
         <v>21</v>
       </c>
       <c r="B1043" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1043"/>
       <c r="D1043"/>
@@ -28627,7 +28627,7 @@
         <v>22</v>
       </c>
       <c r="B1044" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1044"/>
       <c r="D1044"/>
@@ -28654,7 +28654,7 @@
         <v>23</v>
       </c>
       <c r="B1045" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1045"/>
       <c r="D1045"/>
@@ -28679,7 +28679,7 @@
         <v>24</v>
       </c>
       <c r="B1046" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1046"/>
       <c r="D1046"/>
@@ -28706,7 +28706,7 @@
         <v>25</v>
       </c>
       <c r="B1047" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1047"/>
       <c r="D1047"/>
@@ -28731,7 +28731,7 @@
         <v>26</v>
       </c>
       <c r="B1048" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1048"/>
       <c r="D1048"/>
@@ -28756,7 +28756,7 @@
         <v>27</v>
       </c>
       <c r="B1049" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1049"/>
       <c r="D1049"/>
@@ -28783,7 +28783,7 @@
         <v>28</v>
       </c>
       <c r="B1050" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1050"/>
       <c r="D1050"/>
@@ -28810,7 +28810,7 @@
         <v>29</v>
       </c>
       <c r="B1051" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1051"/>
       <c r="D1051"/>
@@ -28837,7 +28837,7 @@
         <v>30</v>
       </c>
       <c r="B1052" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1052"/>
       <c r="D1052"/>
@@ -28862,7 +28862,7 @@
         <v>31</v>
       </c>
       <c r="B1053" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1053"/>
       <c r="D1053"/>
@@ -28887,7 +28887,7 @@
         <v>32</v>
       </c>
       <c r="B1054" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1054"/>
       <c r="D1054"/>
@@ -28914,7 +28914,7 @@
         <v>33</v>
       </c>
       <c r="B1055" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1055"/>
       <c r="D1055"/>
@@ -28939,7 +28939,7 @@
         <v>34</v>
       </c>
       <c r="B1056" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1056"/>
       <c r="D1056"/>
@@ -28966,7 +28966,7 @@
         <v>35</v>
       </c>
       <c r="B1057" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1057"/>
       <c r="D1057"/>
@@ -29407,7 +29407,7 @@
         <v>19</v>
       </c>
       <c r="B1074" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1074"/>
       <c r="D1074"/>
@@ -29432,7 +29432,7 @@
         <v>21</v>
       </c>
       <c r="B1075" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1075"/>
       <c r="D1075"/>
@@ -29459,7 +29459,7 @@
         <v>22</v>
       </c>
       <c r="B1076" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1076"/>
       <c r="D1076"/>
@@ -29486,7 +29486,7 @@
         <v>23</v>
       </c>
       <c r="B1077" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1077"/>
       <c r="D1077"/>
@@ -29511,7 +29511,7 @@
         <v>24</v>
       </c>
       <c r="B1078" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1078"/>
       <c r="D1078"/>
@@ -29538,7 +29538,7 @@
         <v>25</v>
       </c>
       <c r="B1079" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1079"/>
       <c r="D1079"/>
@@ -29563,7 +29563,7 @@
         <v>26</v>
       </c>
       <c r="B1080" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1080"/>
       <c r="D1080"/>
@@ -29588,7 +29588,7 @@
         <v>27</v>
       </c>
       <c r="B1081" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1081"/>
       <c r="D1081"/>
@@ -29615,7 +29615,7 @@
         <v>28</v>
       </c>
       <c r="B1082" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1082"/>
       <c r="D1082"/>
@@ -29642,7 +29642,7 @@
         <v>29</v>
       </c>
       <c r="B1083" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1083"/>
       <c r="D1083"/>
@@ -29669,7 +29669,7 @@
         <v>30</v>
       </c>
       <c r="B1084" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1084"/>
       <c r="D1084"/>
@@ -29694,7 +29694,7 @@
         <v>31</v>
       </c>
       <c r="B1085" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1085"/>
       <c r="D1085"/>
@@ -29719,7 +29719,7 @@
         <v>32</v>
       </c>
       <c r="B1086" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1086"/>
       <c r="D1086"/>
@@ -29746,7 +29746,7 @@
         <v>33</v>
       </c>
       <c r="B1087" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1087"/>
       <c r="D1087"/>
@@ -29771,7 +29771,7 @@
         <v>34</v>
       </c>
       <c r="B1088" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1088"/>
       <c r="D1088"/>
@@ -29798,7 +29798,7 @@
         <v>35</v>
       </c>
       <c r="B1089" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C1089"/>
       <c r="D1089"/>
@@ -29823,7 +29823,7 @@
         <v>19</v>
       </c>
       <c r="B1090" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1090"/>
       <c r="D1090"/>
@@ -29850,7 +29850,7 @@
         <v>21</v>
       </c>
       <c r="B1091" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1091"/>
       <c r="D1091"/>
@@ -29875,7 +29875,7 @@
         <v>22</v>
       </c>
       <c r="B1092" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1092"/>
       <c r="D1092"/>
@@ -29900,7 +29900,7 @@
         <v>23</v>
       </c>
       <c r="B1093" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1093"/>
       <c r="D1093"/>
@@ -29927,7 +29927,7 @@
         <v>24</v>
       </c>
       <c r="B1094" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1094"/>
       <c r="D1094"/>
@@ -29952,7 +29952,7 @@
         <v>25</v>
       </c>
       <c r="B1095" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1095"/>
       <c r="D1095"/>
@@ -29979,7 +29979,7 @@
         <v>26</v>
       </c>
       <c r="B1096" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1096"/>
       <c r="D1096"/>
@@ -30006,7 +30006,7 @@
         <v>27</v>
       </c>
       <c r="B1097" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1097"/>
       <c r="D1097"/>
@@ -30031,7 +30031,7 @@
         <v>28</v>
       </c>
       <c r="B1098" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1098"/>
       <c r="D1098"/>
@@ -30056,7 +30056,7 @@
         <v>29</v>
       </c>
       <c r="B1099" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1099"/>
       <c r="D1099"/>
@@ -30081,7 +30081,7 @@
         <v>30</v>
       </c>
       <c r="B1100" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1100"/>
       <c r="D1100"/>
@@ -30108,7 +30108,7 @@
         <v>31</v>
       </c>
       <c r="B1101" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1101"/>
       <c r="D1101"/>
@@ -30135,7 +30135,7 @@
         <v>32</v>
       </c>
       <c r="B1102" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1102"/>
       <c r="D1102"/>
@@ -30160,7 +30160,7 @@
         <v>33</v>
       </c>
       <c r="B1103" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1103"/>
       <c r="D1103"/>
@@ -30187,7 +30187,7 @@
         <v>34</v>
       </c>
       <c r="B1104" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1104"/>
       <c r="D1104"/>
@@ -30212,7 +30212,7 @@
         <v>35</v>
       </c>
       <c r="B1105" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C1105"/>
       <c r="D1105"/>
@@ -30239,7 +30239,7 @@
         <v>19</v>
       </c>
       <c r="B1106" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1106"/>
       <c r="D1106"/>
@@ -30266,7 +30266,7 @@
         <v>21</v>
       </c>
       <c r="B1107" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1107"/>
       <c r="D1107"/>
@@ -30291,7 +30291,7 @@
         <v>22</v>
       </c>
       <c r="B1108" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1108"/>
       <c r="D1108"/>
@@ -30316,7 +30316,7 @@
         <v>23</v>
       </c>
       <c r="B1109" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1109"/>
       <c r="D1109"/>
@@ -30343,7 +30343,7 @@
         <v>24</v>
       </c>
       <c r="B1110" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1110"/>
       <c r="D1110"/>
@@ -30368,7 +30368,7 @@
         <v>25</v>
       </c>
       <c r="B1111" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1111"/>
       <c r="D1111"/>
@@ -30395,7 +30395,7 @@
         <v>26</v>
       </c>
       <c r="B1112" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1112"/>
       <c r="D1112"/>
@@ -30422,7 +30422,7 @@
         <v>27</v>
       </c>
       <c r="B1113" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1113"/>
       <c r="D1113"/>
@@ -30447,7 +30447,7 @@
         <v>28</v>
       </c>
       <c r="B1114" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1114"/>
       <c r="D1114"/>
@@ -30472,7 +30472,7 @@
         <v>29</v>
       </c>
       <c r="B1115" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1115"/>
       <c r="D1115"/>
@@ -30497,7 +30497,7 @@
         <v>30</v>
       </c>
       <c r="B1116" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1116"/>
       <c r="D1116"/>
@@ -30524,7 +30524,7 @@
         <v>31</v>
       </c>
       <c r="B1117" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1117"/>
       <c r="D1117"/>
@@ -30551,7 +30551,7 @@
         <v>32</v>
       </c>
       <c r="B1118" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1118"/>
       <c r="D1118"/>
@@ -30576,7 +30576,7 @@
         <v>33</v>
       </c>
       <c r="B1119" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1119"/>
       <c r="D1119"/>
@@ -30603,7 +30603,7 @@
         <v>34</v>
       </c>
       <c r="B1120" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1120"/>
       <c r="D1120"/>
@@ -30628,7 +30628,7 @@
         <v>35</v>
       </c>
       <c r="B1121" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C1121"/>
       <c r="D1121"/>
@@ -30655,7 +30655,7 @@
         <v>19</v>
       </c>
       <c r="B1122" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1122"/>
       <c r="D1122"/>
@@ -30682,7 +30682,7 @@
         <v>21</v>
       </c>
       <c r="B1123" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1123"/>
       <c r="D1123"/>
@@ -30707,7 +30707,7 @@
         <v>22</v>
       </c>
       <c r="B1124" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1124"/>
       <c r="D1124"/>
@@ -30732,7 +30732,7 @@
         <v>23</v>
       </c>
       <c r="B1125" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1125"/>
       <c r="D1125"/>
@@ -30759,7 +30759,7 @@
         <v>24</v>
       </c>
       <c r="B1126" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1126"/>
       <c r="D1126"/>
@@ -30784,7 +30784,7 @@
         <v>25</v>
       </c>
       <c r="B1127" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1127"/>
       <c r="D1127"/>
@@ -30811,7 +30811,7 @@
         <v>26</v>
       </c>
       <c r="B1128" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1128"/>
       <c r="D1128"/>
@@ -30838,7 +30838,7 @@
         <v>27</v>
       </c>
       <c r="B1129" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1129"/>
       <c r="D1129"/>
@@ -30863,7 +30863,7 @@
         <v>28</v>
       </c>
       <c r="B1130" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1130"/>
       <c r="D1130"/>
@@ -30888,7 +30888,7 @@
         <v>29</v>
       </c>
       <c r="B1131" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1131"/>
       <c r="D1131"/>
@@ -30913,7 +30913,7 @@
         <v>30</v>
       </c>
       <c r="B1132" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1132"/>
       <c r="D1132"/>
@@ -30940,7 +30940,7 @@
         <v>31</v>
       </c>
       <c r="B1133" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1133"/>
       <c r="D1133"/>
@@ -30967,7 +30967,7 @@
         <v>32</v>
       </c>
       <c r="B1134" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1134"/>
       <c r="D1134"/>
@@ -30992,7 +30992,7 @@
         <v>33</v>
       </c>
       <c r="B1135" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1135"/>
       <c r="D1135"/>
@@ -31019,7 +31019,7 @@
         <v>34</v>
       </c>
       <c r="B1136" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1136"/>
       <c r="D1136"/>
@@ -31044,7 +31044,7 @@
         <v>35</v>
       </c>
       <c r="B1137" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1137"/>
       <c r="D1137"/>
@@ -31487,7 +31487,7 @@
         <v>19</v>
       </c>
       <c r="B1154" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1154"/>
       <c r="D1154"/>
@@ -31514,7 +31514,7 @@
         <v>21</v>
       </c>
       <c r="B1155" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1155"/>
       <c r="D1155"/>
@@ -31539,7 +31539,7 @@
         <v>22</v>
       </c>
       <c r="B1156" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1156"/>
       <c r="D1156"/>
@@ -31564,7 +31564,7 @@
         <v>23</v>
       </c>
       <c r="B1157" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1157"/>
       <c r="D1157"/>
@@ -31591,7 +31591,7 @@
         <v>24</v>
       </c>
       <c r="B1158" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1158"/>
       <c r="D1158"/>
@@ -31616,7 +31616,7 @@
         <v>25</v>
       </c>
       <c r="B1159" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1159"/>
       <c r="D1159"/>
@@ -31643,7 +31643,7 @@
         <v>26</v>
       </c>
       <c r="B1160" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1160"/>
       <c r="D1160"/>
@@ -31670,7 +31670,7 @@
         <v>27</v>
       </c>
       <c r="B1161" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1161"/>
       <c r="D1161"/>
@@ -31695,7 +31695,7 @@
         <v>28</v>
       </c>
       <c r="B1162" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1162"/>
       <c r="D1162"/>
@@ -31720,7 +31720,7 @@
         <v>29</v>
       </c>
       <c r="B1163" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1163"/>
       <c r="D1163"/>
@@ -31745,7 +31745,7 @@
         <v>30</v>
       </c>
       <c r="B1164" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1164"/>
       <c r="D1164"/>
@@ -31772,7 +31772,7 @@
         <v>31</v>
       </c>
       <c r="B1165" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1165"/>
       <c r="D1165"/>
@@ -31799,7 +31799,7 @@
         <v>32</v>
       </c>
       <c r="B1166" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1166"/>
       <c r="D1166"/>
@@ -31824,7 +31824,7 @@
         <v>33</v>
       </c>
       <c r="B1167" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1167"/>
       <c r="D1167"/>
@@ -31851,7 +31851,7 @@
         <v>34</v>
       </c>
       <c r="B1168" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1168"/>
       <c r="D1168"/>
@@ -31876,7 +31876,7 @@
         <v>35</v>
       </c>
       <c r="B1169" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C1169"/>
       <c r="D1169"/>
@@ -31903,7 +31903,7 @@
         <v>19</v>
       </c>
       <c r="B1170" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1170"/>
       <c r="D1170"/>
@@ -31930,7 +31930,7 @@
         <v>21</v>
       </c>
       <c r="B1171" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1171"/>
       <c r="D1171"/>
@@ -31955,7 +31955,7 @@
         <v>22</v>
       </c>
       <c r="B1172" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1172"/>
       <c r="D1172"/>
@@ -31980,7 +31980,7 @@
         <v>23</v>
       </c>
       <c r="B1173" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1173"/>
       <c r="D1173"/>
@@ -32007,7 +32007,7 @@
         <v>24</v>
       </c>
       <c r="B1174" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1174"/>
       <c r="D1174"/>
@@ -32032,7 +32032,7 @@
         <v>25</v>
       </c>
       <c r="B1175" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1175"/>
       <c r="D1175"/>
@@ -32059,7 +32059,7 @@
         <v>26</v>
       </c>
       <c r="B1176" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1176"/>
       <c r="D1176"/>
@@ -32086,7 +32086,7 @@
         <v>27</v>
       </c>
       <c r="B1177" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1177"/>
       <c r="D1177"/>
@@ -32111,7 +32111,7 @@
         <v>28</v>
       </c>
       <c r="B1178" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1178"/>
       <c r="D1178"/>
@@ -32136,7 +32136,7 @@
         <v>29</v>
       </c>
       <c r="B1179" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1179"/>
       <c r="D1179"/>
@@ -32161,7 +32161,7 @@
         <v>30</v>
       </c>
       <c r="B1180" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1180"/>
       <c r="D1180"/>
@@ -32188,7 +32188,7 @@
         <v>31</v>
       </c>
       <c r="B1181" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1181"/>
       <c r="D1181"/>
@@ -32215,7 +32215,7 @@
         <v>32</v>
       </c>
       <c r="B1182" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1182"/>
       <c r="D1182"/>
@@ -32240,7 +32240,7 @@
         <v>33</v>
       </c>
       <c r="B1183" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1183"/>
       <c r="D1183"/>
@@ -32267,7 +32267,7 @@
         <v>34</v>
       </c>
       <c r="B1184" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1184"/>
       <c r="D1184"/>
@@ -32292,7 +32292,7 @@
         <v>35</v>
       </c>
       <c r="B1185" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C1185"/>
       <c r="D1185"/>
@@ -32727,7 +32727,7 @@
         <v>19</v>
       </c>
       <c r="B1202" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1202"/>
       <c r="D1202"/>
@@ -32754,7 +32754,7 @@
         <v>21</v>
       </c>
       <c r="B1203" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1203"/>
       <c r="D1203"/>
@@ -32781,7 +32781,7 @@
         <v>22</v>
       </c>
       <c r="B1204" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1204"/>
       <c r="D1204"/>
@@ -32808,7 +32808,7 @@
         <v>23</v>
       </c>
       <c r="B1205" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1205"/>
       <c r="D1205"/>
@@ -32835,7 +32835,7 @@
         <v>24</v>
       </c>
       <c r="B1206" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1206"/>
       <c r="D1206"/>
@@ -32862,7 +32862,7 @@
         <v>25</v>
       </c>
       <c r="B1207" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1207"/>
       <c r="D1207"/>
@@ -32889,7 +32889,7 @@
         <v>26</v>
       </c>
       <c r="B1208" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1208"/>
       <c r="D1208"/>
@@ -32916,7 +32916,7 @@
         <v>27</v>
       </c>
       <c r="B1209" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1209"/>
       <c r="D1209"/>
@@ -32943,7 +32943,7 @@
         <v>28</v>
       </c>
       <c r="B1210" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1210"/>
       <c r="D1210"/>
@@ -32970,7 +32970,7 @@
         <v>29</v>
       </c>
       <c r="B1211" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1211"/>
       <c r="D1211"/>
@@ -32997,7 +32997,7 @@
         <v>30</v>
       </c>
       <c r="B1212" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1212"/>
       <c r="D1212"/>
@@ -33024,7 +33024,7 @@
         <v>31</v>
       </c>
       <c r="B1213" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1213"/>
       <c r="D1213"/>
@@ -33051,7 +33051,7 @@
         <v>32</v>
       </c>
       <c r="B1214" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1214"/>
       <c r="D1214"/>
@@ -33078,7 +33078,7 @@
         <v>33</v>
       </c>
       <c r="B1215" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1215"/>
       <c r="D1215"/>
@@ -33105,7 +33105,7 @@
         <v>34</v>
       </c>
       <c r="B1216" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1216"/>
       <c r="D1216"/>
@@ -33132,7 +33132,7 @@
         <v>35</v>
       </c>
       <c r="B1217" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C1217"/>
       <c r="D1217"/>
@@ -33159,7 +33159,7 @@
         <v>19</v>
       </c>
       <c r="B1218" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1218"/>
       <c r="D1218"/>
@@ -33186,7 +33186,7 @@
         <v>21</v>
       </c>
       <c r="B1219" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1219"/>
       <c r="D1219"/>
@@ -33213,7 +33213,7 @@
         <v>22</v>
       </c>
       <c r="B1220" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1220"/>
       <c r="D1220"/>
@@ -33240,7 +33240,7 @@
         <v>23</v>
       </c>
       <c r="B1221" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1221"/>
       <c r="D1221"/>
@@ -33267,7 +33267,7 @@
         <v>24</v>
       </c>
       <c r="B1222" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1222"/>
       <c r="D1222"/>
@@ -33294,7 +33294,7 @@
         <v>25</v>
       </c>
       <c r="B1223" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1223"/>
       <c r="D1223"/>
@@ -33321,7 +33321,7 @@
         <v>26</v>
       </c>
       <c r="B1224" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1224"/>
       <c r="D1224"/>
@@ -33348,7 +33348,7 @@
         <v>27</v>
       </c>
       <c r="B1225" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1225"/>
       <c r="D1225"/>
@@ -33375,7 +33375,7 @@
         <v>28</v>
       </c>
       <c r="B1226" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1226"/>
       <c r="D1226"/>
@@ -33402,7 +33402,7 @@
         <v>29</v>
       </c>
       <c r="B1227" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1227"/>
       <c r="D1227"/>
@@ -33429,7 +33429,7 @@
         <v>30</v>
       </c>
       <c r="B1228" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1228"/>
       <c r="D1228"/>
@@ -33456,7 +33456,7 @@
         <v>31</v>
       </c>
       <c r="B1229" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1229"/>
       <c r="D1229"/>
@@ -33483,7 +33483,7 @@
         <v>32</v>
       </c>
       <c r="B1230" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1230"/>
       <c r="D1230"/>
@@ -33510,7 +33510,7 @@
         <v>33</v>
       </c>
       <c r="B1231" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1231"/>
       <c r="D1231"/>
@@ -33537,7 +33537,7 @@
         <v>34</v>
       </c>
       <c r="B1232" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1232"/>
       <c r="D1232"/>
@@ -33564,7 +33564,7 @@
         <v>35</v>
       </c>
       <c r="B1233" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C1233"/>
       <c r="D1233"/>
@@ -33591,7 +33591,7 @@
         <v>19</v>
       </c>
       <c r="B1234" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1234"/>
       <c r="D1234"/>
@@ -33618,7 +33618,7 @@
         <v>21</v>
       </c>
       <c r="B1235" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1235"/>
       <c r="D1235"/>
@@ -33645,7 +33645,7 @@
         <v>22</v>
       </c>
       <c r="B1236" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1236"/>
       <c r="D1236"/>
@@ -33672,7 +33672,7 @@
         <v>23</v>
       </c>
       <c r="B1237" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1237"/>
       <c r="D1237"/>
@@ -33699,7 +33699,7 @@
         <v>24</v>
       </c>
       <c r="B1238" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1238"/>
       <c r="D1238"/>
@@ -33726,7 +33726,7 @@
         <v>25</v>
       </c>
       <c r="B1239" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1239"/>
       <c r="D1239"/>
@@ -33753,7 +33753,7 @@
         <v>26</v>
       </c>
       <c r="B1240" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1240"/>
       <c r="D1240"/>
@@ -33780,7 +33780,7 @@
         <v>27</v>
       </c>
       <c r="B1241" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1241"/>
       <c r="D1241"/>
@@ -33807,7 +33807,7 @@
         <v>28</v>
       </c>
       <c r="B1242" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1242"/>
       <c r="D1242"/>
@@ -33834,7 +33834,7 @@
         <v>29</v>
       </c>
       <c r="B1243" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1243"/>
       <c r="D1243"/>
@@ -33861,7 +33861,7 @@
         <v>30</v>
       </c>
       <c r="B1244" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1244"/>
       <c r="D1244"/>
@@ -33888,7 +33888,7 @@
         <v>31</v>
       </c>
       <c r="B1245" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1245"/>
       <c r="D1245"/>
@@ -33915,7 +33915,7 @@
         <v>32</v>
       </c>
       <c r="B1246" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1246"/>
       <c r="D1246"/>
@@ -33942,7 +33942,7 @@
         <v>33</v>
       </c>
       <c r="B1247" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1247"/>
       <c r="D1247"/>
@@ -33969,7 +33969,7 @@
         <v>34</v>
       </c>
       <c r="B1248" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1248"/>
       <c r="D1248"/>
@@ -33996,7 +33996,7 @@
         <v>35</v>
       </c>
       <c r="B1249" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1249"/>
       <c r="D1249"/>
@@ -34023,7 +34023,7 @@
         <v>19</v>
       </c>
       <c r="B1250" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1250"/>
       <c r="D1250"/>
@@ -34050,7 +34050,7 @@
         <v>21</v>
       </c>
       <c r="B1251" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1251"/>
       <c r="D1251"/>
@@ -34077,7 +34077,7 @@
         <v>22</v>
       </c>
       <c r="B1252" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1252"/>
       <c r="D1252"/>
@@ -34104,7 +34104,7 @@
         <v>23</v>
       </c>
       <c r="B1253" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1253"/>
       <c r="D1253"/>
@@ -34131,7 +34131,7 @@
         <v>24</v>
       </c>
       <c r="B1254" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1254"/>
       <c r="D1254"/>
@@ -34158,7 +34158,7 @@
         <v>25</v>
       </c>
       <c r="B1255" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1255"/>
       <c r="D1255"/>
@@ -34185,7 +34185,7 @@
         <v>26</v>
       </c>
       <c r="B1256" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1256"/>
       <c r="D1256"/>
@@ -34212,7 +34212,7 @@
         <v>27</v>
       </c>
       <c r="B1257" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1257"/>
       <c r="D1257"/>
@@ -34239,7 +34239,7 @@
         <v>28</v>
       </c>
       <c r="B1258" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1258"/>
       <c r="D1258"/>
@@ -34266,7 +34266,7 @@
         <v>29</v>
       </c>
       <c r="B1259" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1259"/>
       <c r="D1259"/>
@@ -34293,7 +34293,7 @@
         <v>30</v>
       </c>
       <c r="B1260" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1260"/>
       <c r="D1260"/>
@@ -34320,7 +34320,7 @@
         <v>31</v>
       </c>
       <c r="B1261" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1261"/>
       <c r="D1261"/>
@@ -34347,7 +34347,7 @@
         <v>32</v>
       </c>
       <c r="B1262" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1262"/>
       <c r="D1262"/>
@@ -34374,7 +34374,7 @@
         <v>33</v>
       </c>
       <c r="B1263" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1263"/>
       <c r="D1263"/>
@@ -34401,7 +34401,7 @@
         <v>34</v>
       </c>
       <c r="B1264" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1264"/>
       <c r="D1264"/>
@@ -34428,7 +34428,7 @@
         <v>35</v>
       </c>
       <c r="B1265" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1265"/>
       <c r="D1265"/>
@@ -34887,7 +34887,7 @@
         <v>19</v>
       </c>
       <c r="B1282" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1282"/>
       <c r="D1282"/>
@@ -34914,7 +34914,7 @@
         <v>21</v>
       </c>
       <c r="B1283" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1283"/>
       <c r="D1283"/>
@@ -34941,7 +34941,7 @@
         <v>22</v>
       </c>
       <c r="B1284" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1284"/>
       <c r="D1284"/>
@@ -34968,7 +34968,7 @@
         <v>23</v>
       </c>
       <c r="B1285" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1285"/>
       <c r="D1285"/>
@@ -34995,7 +34995,7 @@
         <v>24</v>
       </c>
       <c r="B1286" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1286"/>
       <c r="D1286"/>
@@ -35022,7 +35022,7 @@
         <v>25</v>
       </c>
       <c r="B1287" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1287"/>
       <c r="D1287"/>
@@ -35049,7 +35049,7 @@
         <v>26</v>
       </c>
       <c r="B1288" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1288"/>
       <c r="D1288"/>
@@ -35076,7 +35076,7 @@
         <v>27</v>
       </c>
       <c r="B1289" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1289"/>
       <c r="D1289"/>
@@ -35103,7 +35103,7 @@
         <v>28</v>
       </c>
       <c r="B1290" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1290"/>
       <c r="D1290"/>
@@ -35130,7 +35130,7 @@
         <v>29</v>
       </c>
       <c r="B1291" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1291"/>
       <c r="D1291"/>
@@ -35157,7 +35157,7 @@
         <v>30</v>
       </c>
       <c r="B1292" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1292"/>
       <c r="D1292"/>
@@ -35184,7 +35184,7 @@
         <v>31</v>
       </c>
       <c r="B1293" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1293"/>
       <c r="D1293"/>
@@ -35211,7 +35211,7 @@
         <v>32</v>
       </c>
       <c r="B1294" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1294"/>
       <c r="D1294"/>
@@ -35238,7 +35238,7 @@
         <v>33</v>
       </c>
       <c r="B1295" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1295"/>
       <c r="D1295"/>
@@ -35265,7 +35265,7 @@
         <v>34</v>
       </c>
       <c r="B1296" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1296"/>
       <c r="D1296"/>
@@ -35292,7 +35292,7 @@
         <v>35</v>
       </c>
       <c r="B1297" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C1297"/>
       <c r="D1297"/>
@@ -36615,7 +36615,7 @@
         <v>19</v>
       </c>
       <c r="B1346" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1346"/>
       <c r="D1346"/>
@@ -36642,7 +36642,7 @@
         <v>21</v>
       </c>
       <c r="B1347" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1347"/>
       <c r="D1347"/>
@@ -36669,7 +36669,7 @@
         <v>22</v>
       </c>
       <c r="B1348" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1348"/>
       <c r="D1348"/>
@@ -36696,7 +36696,7 @@
         <v>23</v>
       </c>
       <c r="B1349" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1349"/>
       <c r="D1349"/>
@@ -36723,7 +36723,7 @@
         <v>24</v>
       </c>
       <c r="B1350" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1350"/>
       <c r="D1350"/>
@@ -36750,7 +36750,7 @@
         <v>25</v>
       </c>
       <c r="B1351" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1351"/>
       <c r="D1351"/>
@@ -36777,7 +36777,7 @@
         <v>26</v>
       </c>
       <c r="B1352" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1352"/>
       <c r="D1352"/>
@@ -36804,7 +36804,7 @@
         <v>27</v>
       </c>
       <c r="B1353" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1353"/>
       <c r="D1353"/>
@@ -36831,7 +36831,7 @@
         <v>28</v>
       </c>
       <c r="B1354" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1354"/>
       <c r="D1354"/>
@@ -36858,7 +36858,7 @@
         <v>29</v>
       </c>
       <c r="B1355" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1355"/>
       <c r="D1355"/>
@@ -36885,7 +36885,7 @@
         <v>30</v>
       </c>
       <c r="B1356" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1356"/>
       <c r="D1356"/>
@@ -36912,7 +36912,7 @@
         <v>31</v>
       </c>
       <c r="B1357" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1357"/>
       <c r="D1357"/>
@@ -36939,7 +36939,7 @@
         <v>32</v>
       </c>
       <c r="B1358" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1358"/>
       <c r="D1358"/>
@@ -36966,7 +36966,7 @@
         <v>33</v>
       </c>
       <c r="B1359" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1359"/>
       <c r="D1359"/>
@@ -36993,7 +36993,7 @@
         <v>34</v>
       </c>
       <c r="B1360" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1360"/>
       <c r="D1360"/>
@@ -37020,7 +37020,7 @@
         <v>35</v>
       </c>
       <c r="B1361" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1361"/>
       <c r="D1361"/>
@@ -37047,7 +37047,7 @@
         <v>19</v>
       </c>
       <c r="B1362" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1362"/>
       <c r="D1362"/>
@@ -37074,7 +37074,7 @@
         <v>21</v>
       </c>
       <c r="B1363" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1363"/>
       <c r="D1363"/>
@@ -37101,7 +37101,7 @@
         <v>22</v>
       </c>
       <c r="B1364" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1364"/>
       <c r="D1364"/>
@@ -37128,7 +37128,7 @@
         <v>23</v>
       </c>
       <c r="B1365" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1365"/>
       <c r="D1365"/>
@@ -37155,7 +37155,7 @@
         <v>24</v>
       </c>
       <c r="B1366" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1366"/>
       <c r="D1366"/>
@@ -37182,7 +37182,7 @@
         <v>25</v>
       </c>
       <c r="B1367" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1367"/>
       <c r="D1367"/>
@@ -37209,7 +37209,7 @@
         <v>26</v>
       </c>
       <c r="B1368" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1368"/>
       <c r="D1368"/>
@@ -37236,7 +37236,7 @@
         <v>27</v>
       </c>
       <c r="B1369" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1369"/>
       <c r="D1369"/>
@@ -37263,7 +37263,7 @@
         <v>28</v>
       </c>
       <c r="B1370" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1370"/>
       <c r="D1370"/>
@@ -37290,7 +37290,7 @@
         <v>29</v>
       </c>
       <c r="B1371" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1371"/>
       <c r="D1371"/>
@@ -37317,7 +37317,7 @@
         <v>30</v>
       </c>
       <c r="B1372" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1372"/>
       <c r="D1372"/>
@@ -37344,7 +37344,7 @@
         <v>31</v>
       </c>
       <c r="B1373" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1373"/>
       <c r="D1373"/>
@@ -37371,7 +37371,7 @@
         <v>32</v>
       </c>
       <c r="B1374" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1374"/>
       <c r="D1374"/>
@@ -37398,7 +37398,7 @@
         <v>33</v>
       </c>
       <c r="B1375" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1375"/>
       <c r="D1375"/>
@@ -37425,7 +37425,7 @@
         <v>34</v>
       </c>
       <c r="B1376" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1376"/>
       <c r="D1376"/>
@@ -37452,7 +37452,7 @@
         <v>35</v>
       </c>
       <c r="B1377" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1377"/>
       <c r="D1377"/>
@@ -37911,7 +37911,7 @@
         <v>19</v>
       </c>
       <c r="B1394" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1394"/>
       <c r="D1394"/>
@@ -37938,7 +37938,7 @@
         <v>21</v>
       </c>
       <c r="B1395" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1395"/>
       <c r="D1395"/>
@@ -37965,7 +37965,7 @@
         <v>22</v>
       </c>
       <c r="B1396" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1396"/>
       <c r="D1396"/>
@@ -37992,7 +37992,7 @@
         <v>23</v>
       </c>
       <c r="B1397" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1397"/>
       <c r="D1397"/>
@@ -38019,7 +38019,7 @@
         <v>24</v>
       </c>
       <c r="B1398" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1398"/>
       <c r="D1398"/>
@@ -38046,7 +38046,7 @@
         <v>25</v>
       </c>
       <c r="B1399" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1399"/>
       <c r="D1399"/>
@@ -38073,7 +38073,7 @@
         <v>26</v>
       </c>
       <c r="B1400" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1400"/>
       <c r="D1400"/>
@@ -38100,7 +38100,7 @@
         <v>27</v>
       </c>
       <c r="B1401" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1401"/>
       <c r="D1401"/>
@@ -38127,7 +38127,7 @@
         <v>28</v>
       </c>
       <c r="B1402" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1402"/>
       <c r="D1402"/>
@@ -38154,7 +38154,7 @@
         <v>29</v>
       </c>
       <c r="B1403" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1403"/>
       <c r="D1403"/>
@@ -38181,7 +38181,7 @@
         <v>30</v>
       </c>
       <c r="B1404" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1404"/>
       <c r="D1404"/>
@@ -38208,7 +38208,7 @@
         <v>31</v>
       </c>
       <c r="B1405" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1405"/>
       <c r="D1405"/>
@@ -38235,7 +38235,7 @@
         <v>32</v>
       </c>
       <c r="B1406" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1406"/>
       <c r="D1406"/>
@@ -38262,7 +38262,7 @@
         <v>33</v>
       </c>
       <c r="B1407" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1407"/>
       <c r="D1407"/>
@@ -38289,7 +38289,7 @@
         <v>34</v>
       </c>
       <c r="B1408" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1408"/>
       <c r="D1408"/>
@@ -38316,7 +38316,7 @@
         <v>35</v>
       </c>
       <c r="B1409" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C1409"/>
       <c r="D1409"/>
@@ -38775,7 +38775,7 @@
         <v>19</v>
       </c>
       <c r="B1426" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1426"/>
       <c r="D1426"/>
@@ -38802,7 +38802,7 @@
         <v>21</v>
       </c>
       <c r="B1427" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1427"/>
       <c r="D1427"/>
@@ -38829,7 +38829,7 @@
         <v>22</v>
       </c>
       <c r="B1428" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1428"/>
       <c r="D1428"/>
@@ -38856,7 +38856,7 @@
         <v>23</v>
       </c>
       <c r="B1429" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1429"/>
       <c r="D1429"/>
@@ -38883,7 +38883,7 @@
         <v>24</v>
       </c>
       <c r="B1430" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1430"/>
       <c r="D1430"/>
@@ -38910,7 +38910,7 @@
         <v>25</v>
       </c>
       <c r="B1431" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C1431"/>
       <c r="D1431"/>
@@ -38937,7 +38937,7 @@
         <v>26</v>
       </c>
       <c r="B1432" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1432"/>
       <c r="D1432"/>
@@ -38964,7 +38964,7 @@
         <v>27</v>
       </c>
       <c r="B1433" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1433"/>
       <c r="D1433"/>
@@ -38991,7 +38991,7 @@
         <v>28</v>
       </c>
       <c r="B1434" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1434"/>
       <c r="D1434"/>
@@ -39018,7 +39018,7 @@
         <v>29</v>
       </c>
       <c r="B1435" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1435"/>
       <c r="D1435"/>
@@ -39045,7 +39045,7 @@
         <v>30</v>
       </c>
       <c r="B1436" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1436"/>
       <c r="D1436"/>
@@ -39072,7 +39072,7 @@
         <v>31</v>
       </c>
       <c r="B1437" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1437"/>
       <c r="D1437"/>
@@ -39099,7 +39099,7 @@
         <v>32</v>
       </c>
       <c r="B1438" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1438"/>
       <c r="D1438"/>
@@ -39126,7 +39126,7 @@
         <v>33</v>
       </c>
       <c r="B1439" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1439"/>
       <c r="D1439"/>
@@ -39153,7 +39153,7 @@
         <v>34</v>
       </c>
       <c r="B1440" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C1440"/>
       <c r="D1440"/>
@@ -39180,7 +39180,7 @@
         <v>35</v>
       </c>
       <c r="B1441" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1441"/>
       <c r="D1441"/>
@@ -39207,7 +39207,7 @@
         <v>19</v>
       </c>
       <c r="B1442" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1442"/>
       <c r="D1442"/>
@@ -39261,7 +39261,7 @@
         <v>22</v>
       </c>
       <c r="B1444" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1444"/>
       <c r="D1444"/>
@@ -39288,7 +39288,7 @@
         <v>23</v>
       </c>
       <c r="B1445" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C1445"/>
       <c r="D1445"/>
@@ -39315,7 +39315,7 @@
         <v>24</v>
       </c>
       <c r="B1446" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C1446"/>
       <c r="D1446"/>
@@ -39369,7 +39369,7 @@
         <v>26</v>
       </c>
       <c r="B1448" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C1448"/>
       <c r="D1448"/>
@@ -39396,7 +39396,7 @@
         <v>27</v>
       </c>
       <c r="B1449" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C1449"/>
       <c r="D1449"/>
@@ -39423,7 +39423,7 @@
         <v>28</v>
       </c>
       <c r="B1450" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C1450"/>
       <c r="D1450"/>
@@ -39450,7 +39450,7 @@
         <v>29</v>
       </c>
       <c r="B1451" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C1451"/>
       <c r="D1451"/>
@@ -39477,7 +39477,7 @@
         <v>30</v>
       </c>
       <c r="B1452" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1452"/>
       <c r="D1452"/>
@@ -39504,7 +39504,7 @@
         <v>31</v>
       </c>
       <c r="B1453" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C1453"/>
       <c r="D1453"/>
@@ -39531,7 +39531,7 @@
         <v>32</v>
       </c>
       <c r="B1454" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="C1454"/>
       <c r="D1454"/>
@@ -39558,7 +39558,7 @@
         <v>33</v>
       </c>
       <c r="B1455" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="C1455"/>
       <c r="D1455"/>
@@ -39585,7 +39585,7 @@
         <v>34</v>
       </c>
       <c r="B1456" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C1456"/>
       <c r="D1456"/>
@@ -39639,7 +39639,7 @@
         <v>19</v>
       </c>
       <c r="B1458" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1458"/>
       <c r="D1458"/>
@@ -39666,7 +39666,7 @@
         <v>21</v>
       </c>
       <c r="B1459" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="C1459"/>
       <c r="D1459"/>
@@ -39693,7 +39693,7 @@
         <v>22</v>
       </c>
       <c r="B1460" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1460"/>
       <c r="D1460"/>
@@ -39720,7 +39720,7 @@
         <v>23</v>
       </c>
       <c r="B1461" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="C1461"/>
       <c r="D1461"/>
@@ -39747,7 +39747,7 @@
         <v>24</v>
       </c>
       <c r="B1462" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="C1462"/>
       <c r="D1462"/>
@@ -39774,7 +39774,7 @@
         <v>25</v>
       </c>
       <c r="B1463" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1463"/>
       <c r="D1463"/>
@@ -39801,7 +39801,7 @@
         <v>26</v>
       </c>
       <c r="B1464" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1464"/>
       <c r="D1464"/>
@@ -39828,7 +39828,7 @@
         <v>27</v>
       </c>
       <c r="B1465" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C1465"/>
       <c r="D1465"/>
@@ -39855,7 +39855,7 @@
         <v>28</v>
       </c>
       <c r="B1466" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1466"/>
       <c r="D1466"/>
@@ -39882,7 +39882,7 @@
         <v>29</v>
       </c>
       <c r="B1467" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="C1467"/>
       <c r="D1467"/>
@@ -39909,7 +39909,7 @@
         <v>30</v>
       </c>
       <c r="B1468" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C1468"/>
       <c r="D1468"/>
@@ -39936,7 +39936,7 @@
         <v>31</v>
       </c>
       <c r="B1469" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1469"/>
       <c r="D1469"/>
@@ -39963,7 +39963,7 @@
         <v>32</v>
       </c>
       <c r="B1470" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C1470"/>
       <c r="D1470"/>
@@ -39990,7 +39990,7 @@
         <v>33</v>
       </c>
       <c r="B1471" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1471"/>
       <c r="D1471"/>
@@ -40017,7 +40017,7 @@
         <v>34</v>
       </c>
       <c r="B1472" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1472"/>
       <c r="D1472"/>
@@ -40044,7 +40044,7 @@
         <v>35</v>
       </c>
       <c r="B1473" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="C1473"/>
       <c r="D1473"/>

</xml_diff>